<commit_message>
funciones 1, 7, 8, 9 xd
</commit_message>
<xml_diff>
--- a/clima.xlsx
+++ b/clima.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
@@ -644,6 +644,114 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Belarus</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Minsk</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="D7" t="n">
+        <v>226</v>
+      </c>
+      <c r="E7" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>dia</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Oeste</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Muy nublado</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Lima</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="D8" t="n">
+        <v>155</v>
+      </c>
+      <c r="E8" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>noche</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Sur</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Muy nublado</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Lima</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="D9" t="n">
+        <v>155</v>
+      </c>
+      <c r="E9" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>noche</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Sur</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Muy nublado</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>